<commit_message>
test: Mo phong dien form e2e va xac thuc du lieu excel thanh cong
</commit_message>
<xml_diff>
--- a/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
+++ b/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
@@ -106,7 +106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -128,11 +128,44 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,6 +201,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -533,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -781,6 +815,237 @@
       <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Cảm ơn anh Việt rất nhiều, nhờ anh mà em tự tin bấm máy quay ngay ngày hôm sau!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0004</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 07:01:36</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Offline Thực Chiến K12 - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Thu Trang</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Quản lý pháp chế MEDLATEC (Chuẩn bị mở cty luật riêng)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://facebook.com/thutrang.law</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>TikTok Video</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định đăng ký chỉ sau 20 giây xem video anh Việt nói về băm nhỏ phân cảnh và ứng dụng AI đa ngành</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Tư duy rất mới về ứng dụng AI, kỹ năng quay dựng và cách làm marketing đa ngành. Tự tin và định hướng rõ ràng hơn rất nhiều.</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>- Cần kiểm soát danh sách check-in vào lớp chặt chẽ hơn
+- Gửi link khảo sát ngắn trước buổi học
+- Thăm hỏi học viên vắng mặt hoặc về sớm
+- Dành 10p cuối giới thiệu gói nâng cao kèm ưu đãi tại lớp
+- Tư vấn rõ ưu đãi giảm 10% khi đăng ký nhóm 2 người</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>AI Chuyên Sâu Tự Động Hóa Video, Xây Kênh Thương Hiệu Cá Nhân</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Zalo</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Giá trị Thầy mang lại là điều vô giá đối với Em ạ! Chúc Thầy và đội ngũ luôn giữ ngọn lửa nhiệt huyết.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0005</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 07:01:36</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Offline Thực Chiến K12 - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Trần Quốc Huy</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Chủ chuỗi thời trang nam tại Hải Phòng</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://tiktok.com/@huytran.menswear</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Facebook Reels / Post</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Video bóc tách kịch bản 3 tầng bán quần áo không bị flop</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Nắm vững kỹ thuật setup 2 máy quay và cách nói chuyện tự nhiên trước ống kính</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>- Mong muốn có thêm buổi thực hành bối cảnh ngoại cảnh
+- Khâu tài liệu phát tay nên in sớm hơn</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Video Ads Bán Hàng Chuyển Đổi Cao</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Zalo</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>Cảm ơn anh Việt nhiều, về Hải Phòng em sẽ bắt tay bấm máy quay ngay loạt video đầu tiên!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0006</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 07:01:36</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Online Video Masterclass K05</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Minh</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>0905123456</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Môi giới Bất động sản cao cấp TP.HCM</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://youtube.com/@hoangminh.batdongsan</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>YouTube Video / Shorts</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Video hướng dẫn làm video BĐS không cần máy xịn, chỉ cần điện thoại và đèn</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Biết cách làm kịch bản đánh trúng nỗi đau người mua nhà và quy trình dựng video nhanh trong 15 phút</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>- Buổi Zoom nên tăng thêm thời lượng hỏi đáp 1-1
+- Gói nâng cao nên có nhóm hỗ trợ sửa video hàng tuần</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>AI Chuyên Sâu Tự Động Hóa Video, Kèm 1-1 Setup Studio &amp; Thực Chiến</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Telegram</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Mong anh sớm mở workshop trực tiếp tại Sài Gòn để anh em trong Nam được gặp anh!</t>
         </is>
       </c>
     </row>
@@ -820,36 +1085,36 @@
           <t>Tổng Số Phản Hồi</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n"/>
+      <c r="B3" s="13" t="n"/>
       <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Điểm Hài Lòng Trung Bình (NPS)</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n"/>
+      <c r="D3" s="13" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Tỷ Lệ Quan Tâm Nâng Cao</t>
         </is>
       </c>
-      <c r="F3" s="7" t="n"/>
+      <c r="F3" s="13" t="n"/>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="8">
         <f>COUNTA('Dữ Liệu Khảo Sát'!A2:A1000)</f>
         <v/>
       </c>
-      <c r="B4" s="7" t="n"/>
+      <c r="B4" s="13" t="n"/>
       <c r="C4" s="9">
         <f>AVERAGE('Dữ Liệu Khảo Sát'!L2:L1000)</f>
         <v/>
       </c>
-      <c r="D4" s="7" t="n"/>
+      <c r="D4" s="13" t="n"/>
       <c r="E4" s="10">
         <f>COUNTIF('Dữ Liệu Khảo Sát'!M2:M1000, "*AI*")/COUNTA('Dữ Liệu Khảo Sát'!A2:A1000)</f>
         <v/>
       </c>
-      <c r="F4" s="7" t="n"/>
+      <c r="F4" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -871,7 +1136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -990,6 +1255,111 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Thu Trang</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Quản lý pháp chế MEDLATEC (Chuẩn bị mở cty luật riêng)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://facebook.com/thutrang.law</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Gói quà Prompt AI + AI Chuyên Sâu Tự Động Hóa Video, Xây Kênh Thương Hiệu Cá Nhân</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Đã tự động gắn tag &amp; sẵn sàng gửi quà Zalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Trần Quốc Huy</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Chủ chuỗi thời trang nam tại Hải Phòng</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://tiktok.com/@huytran.menswear</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Gói quà Prompt AI + Video Ads Bán Hàng Chuyển Đổi Cao</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Đã tự động gắn tag &amp; sẵn sàng gửi quà Zalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Lê Hoàng Minh</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Môi giới Bất động sản cao cấp TP.HCM</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://youtube.com/@hoangminh.batdongsan</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>0905123456</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Gói quà Prompt AI + AI Chuyên Sâu Tự Động Hóa Video, Kèm 1-1 Setup Studio &amp; Thực Chiến</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Đã tự động gắn tag &amp; sẵn sàng gửi quà Zalo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Await client dispatch Telegram NOVA va toi uu nen anh 800px sieu nhe
</commit_message>
<xml_diff>
--- a/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
+++ b/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -694,6 +694,66 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 18:04:24</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Lớp Offline Thực Chiến - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Trần Tuấn Anh (Test Kiểm Thử 100%)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0912888999</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Giám đốc công ty du lịch. Muốn quay video review tour trải nghiệm và chia sẻ mẹo du lịch.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://tiktok.com/@tuananh_travel
+https://facebook.com/tuananhtravel</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Xem video băm kịch bản 3 tầng, thấy thực tế quá nên nhắn tin và đăng ký.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2 ngày học cực kỳ đáng giá, vỡ ra cách tư duy kịch bản và cách cầm máy tự tin.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>2 ảnh</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>📁 Link Drive: https://docs.google.com/spreadsheets/d/15zgMk-Xow8E_Ha1qgWbGtgWEYwygXyAMqFxkczghokM/edit
+1. anh_lop_hoc_1.jpg (195 KB)
+2. anh_lop_hoc_2.jpg (210 KB)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -705,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -826,6 +886,42 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Trần Tuấn Anh</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0912888999</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Du lịch &amp; Tour trải nghiệm</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>tiktok.com/@tuananh_travel
+facebook.com/tuananhtravel</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2 ảnh</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>✅ Đã lưu Zalo, đã bấm follow kênh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Tich hop Google Apps Script Webhook cua anh Viet vao he thong va client form submit
</commit_message>
<xml_diff>
--- a/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
+++ b/Mau_Bang_Khao_Sat_Hoc_Vien_VietMac.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -754,6 +754,124 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 18:21:02</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Lớp Offline Thực Chiến - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Phạm Hoàng Long (Test Persistent 100%)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>0933555777</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Kinh doanh thiết bị điện tử thông minh. Muốn quay video so sánh tính năng và unbox sản phẩm.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://tiktok.com/@hoanglong.tech
+https://youtube.com/@hoanglongreview</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Xem video bóc 3 tầng trên Reels, thấy quá chân thực.</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Lớp học thực chiến chất lượng, thực hành cầm máy quay rất trực quan.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>1 ảnh</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>📁 Link Drive: https://docs.google.com/spreadsheets/d/1J9ZrjLxTba9R-wuet1n_J_hKcL0PVtQDD_ag65Ewx04/edit
+1. anh_thuc_hanh_quay.jpg (80 KB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KS-2026-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>24/08/2026 18:22:09</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Lớp Offline Thực Chiến - Hà Nội</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Nguyễn Hoàng Nam (Test Trình Duyệt Thật)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>0966888999</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Chủ chuỗi nha khoa thẩm mỹ tại Hà Nội. Muốn xây kênh chia sẻ kiến thức nha khoa không đau và bọc sứ thẩm mỹ. Đang bí phần hook 3s đầu.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>https://tiktok.com/@nam.nhakhoa
+https://facebook.com/namdental.clinic</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Lướt thấy video anh chia sẻ bóc kịch bản 3 tầng trên TikTok. Xem cuốn quá nên xem tiếp 4 video rồi nhắn tin đăng ký chuyển khoản luôn.</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>2 ngày học rất đã, vỡ ra cách setup 2 góc máy và tư duy băm cảnh. Hôm nào rảnh em mời anh ly cafe nhé!</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>1 ảnh</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>📁 Link Drive: https://docs.google.com/spreadsheets/d/1J9ZrjLxTba9R-wuet1n_J_hKcL0PVtQDD_ag65Ewx04/edit
+1. anh_chup_lop_hoc_test.jpg (82 KB)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -765,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -922,6 +1040,78 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Phạm Hoàng Long</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0933555777</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Điện tử thông minh &amp; Unbox</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>tiktok.com/@hoanglong.tech
+youtube.com/@hoanglongreview</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1 ảnh</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>✅ Đã lưu Zalo, đã bấm follow kênh</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Hoàng Nam</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0966888999</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Nha khoa thẩm mỹ &amp; Răng sứ</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>tiktok.com/@nam.nhakhoa
+facebook.com/namdental.clinic</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1 ảnh</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>✅ Đã lưu Zalo, đã bấm follow kênh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>